<commit_message>
Restore Spatial Transcriptomics FISH (stx_fish) technology
Re-adds the image-based ST-FISH option to the v0.4 schema so it reappears
in the Technology dropdown. Restores the imaging_protocol component,
is_pathological allowed_values column, three version_*_stx_fish columns,
and the DwC/MIxS/ToL checklists. Regenerates the dist/ manifests.

Co-Authored-By: Claude Opus 4.7 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/dist/checklists/xlsx/dwc/single_cell_manifest_version_dwc_sc_rnaseq_v0.4.xlsx
+++ b/dist/checklists/xlsx/dwc/single_cell_manifest_version_dwc_sc_rnaseq_v0.4.xlsx
@@ -2505,7 +2505,7 @@
       </c>
     </row>
   </sheetData>
-  <sheetProtection password="D553" sheet="1" objects="1" scenarios="1"/>
+  <sheetProtection password="9D13" sheet="1" objects="1" scenarios="1"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
@@ -5586,7 +5586,7 @@
       <c r="A1005" s="7"/>
     </row>
   </sheetData>
-  <sheetProtection password="9067" sheet="1" objects="1" scenarios="1"/>
+  <sheetProtection password="DFB2" sheet="1" objects="1" scenarios="1"/>
   <mergeCells count="1">
     <mergeCell ref="A4:E4"/>
   </mergeCells>
@@ -8793,7 +8793,7 @@
       <c r="A1005" s="7"/>
     </row>
   </sheetData>
-  <sheetProtection password="9643" sheet="1" objects="1" scenarios="1"/>
+  <sheetProtection password="F095" sheet="1" objects="1" scenarios="1"/>
   <mergeCells count="1">
     <mergeCell ref="A4:O4"/>
   </mergeCells>
@@ -11869,7 +11869,7 @@
       <c r="A1005" s="7"/>
     </row>
   </sheetData>
-  <sheetProtection password="AA59" sheet="1" objects="1" scenarios="1"/>
+  <sheetProtection password="EA60" sheet="1" objects="1" scenarios="1"/>
   <mergeCells count="1">
     <mergeCell ref="A4:D4"/>
   </mergeCells>
@@ -11988,7 +11988,7 @@
       <c r="H4" s="6"/>
     </row>
   </sheetData>
-  <sheetProtection password="A515" sheet="1" objects="1" scenarios="1"/>
+  <sheetProtection password="B275" sheet="1" objects="1" scenarios="1"/>
   <mergeCells count="1">
     <mergeCell ref="A4:H4"/>
   </mergeCells>
@@ -18143,7 +18143,7 @@
       <c r="D1005" s="7"/>
     </row>
   </sheetData>
-  <sheetProtection password="DF5B" sheet="1" objects="1" scenarios="1"/>
+  <sheetProtection password="D7F8" sheet="1" objects="1" scenarios="1"/>
   <mergeCells count="1">
     <mergeCell ref="A4:K4"/>
   </mergeCells>
@@ -22354,7 +22354,7 @@
       <c r="B1005" s="7"/>
     </row>
   </sheetData>
-  <sheetProtection password="F7A3" sheet="1" objects="1" scenarios="1"/>
+  <sheetProtection password="C4D9" sheet="1" objects="1" scenarios="1"/>
   <mergeCells count="1">
     <mergeCell ref="A4:P4"/>
   </mergeCells>
@@ -28526,7 +28526,7 @@
       <c r="D1005" s="7"/>
     </row>
   </sheetData>
-  <sheetProtection password="ED24" sheet="1" objects="1" scenarios="1"/>
+  <sheetProtection password="8403" sheet="1" objects="1" scenarios="1"/>
   <mergeCells count="1">
     <mergeCell ref="A4:K4"/>
   </mergeCells>
@@ -28650,7 +28650,7 @@
       <c r="H4" s="6"/>
     </row>
   </sheetData>
-  <sheetProtection password="90C3" sheet="1" objects="1" scenarios="1"/>
+  <sheetProtection password="835F" sheet="1" objects="1" scenarios="1"/>
   <mergeCells count="1">
     <mergeCell ref="A4:H4"/>
   </mergeCells>
@@ -32436,7 +32436,7 @@
       <c r="A1005" s="7"/>
     </row>
   </sheetData>
-  <sheetProtection password="CF19" sheet="1" objects="1" scenarios="1"/>
+  <sheetProtection password="E1BB" sheet="1" objects="1" scenarios="1"/>
   <mergeCells count="1">
     <mergeCell ref="A4:H4"/>
   </mergeCells>
@@ -36526,7 +36526,7 @@
       <c r="B1005" s="7"/>
     </row>
   </sheetData>
-  <sheetProtection password="996A" sheet="1" objects="1" scenarios="1"/>
+  <sheetProtection password="C78A" sheet="1" objects="1" scenarios="1"/>
   <mergeCells count="1">
     <mergeCell ref="A4:E4"/>
   </mergeCells>
@@ -40682,7 +40682,7 @@
       <c r="B1005" s="7"/>
     </row>
   </sheetData>
-  <sheetProtection password="F3FA" sheet="1" objects="1" scenarios="1"/>
+  <sheetProtection password="D8A3" sheet="1" objects="1" scenarios="1"/>
   <mergeCells count="1">
     <mergeCell ref="A4:K4"/>
   </mergeCells>
@@ -46878,7 +46878,7 @@
       <c r="D1005" s="7"/>
     </row>
   </sheetData>
-  <sheetProtection password="EF34" sheet="1" objects="1" scenarios="1"/>
+  <sheetProtection password="C3E4" sheet="1" objects="1" scenarios="1"/>
   <mergeCells count="1">
     <mergeCell ref="A4:N4"/>
   </mergeCells>
@@ -52249,7 +52249,7 @@
       <c r="C1005" s="7"/>
     </row>
   </sheetData>
-  <sheetProtection password="EAFE" sheet="1" objects="1" scenarios="1"/>
+  <sheetProtection password="A565" sheet="1" objects="1" scenarios="1"/>
   <mergeCells count="1">
     <mergeCell ref="A4:AD4"/>
   </mergeCells>
@@ -56469,7 +56469,7 @@
       <c r="B1005" s="7"/>
     </row>
   </sheetData>
-  <sheetProtection password="A4F0" sheet="1" objects="1" scenarios="1"/>
+  <sheetProtection password="DEAA" sheet="1" objects="1" scenarios="1"/>
   <mergeCells count="1">
     <mergeCell ref="A4:N4"/>
   </mergeCells>

</xml_diff>

<commit_message>
Add image data - STX FISH & REMBI
- Spatial Transcriptomics (FISH) image metadata was added in addition to REMBI
- Code was modularised to improve reusability
- Related commits: eb6f1d4, 24e965f
</commit_message>
<xml_diff>
--- a/dist/checklists/xlsx/dwc/single_cell_manifest_version_dwc_sc_rnaseq_v0.4.xlsx
+++ b/dist/checklists/xlsx/dwc/single_cell_manifest_version_dwc_sc_rnaseq_v0.4.xlsx
@@ -52,7 +52,7 @@
     <t>version_dwc_sc_rnaseq</t>
   </si>
   <si>
-    <t>Single-cell Ribonucleic Acid Sequencing Sequencing [Darwin Core]</t>
+    <t>Single-cell Ribonucleic Acid Sequencing [Darwin Core]</t>
   </si>
   <si>
     <t>For single-cell Ribonucleic Acid Sequencing (RNA-seq)  studies aimed focused on biodiversity-related information in alignment with the Darwin Core (DwC) standard.</t>
@@ -2457,7 +2457,7 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="21.85546875" style="1" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="59.42578125" style="1" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="48.7109375" style="1" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="146.5703125" style="1" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="8.7109375" style="1" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="10.85546875" style="1" bestFit="1" customWidth="1"/>
@@ -2505,7 +2505,7 @@
       </c>
     </row>
   </sheetData>
-  <sheetProtection password="D553" sheet="1" objects="1" scenarios="1"/>
+  <sheetProtection password="B153" sheet="1" objects="1" scenarios="1"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
@@ -5586,7 +5586,7 @@
       <c r="A1005" s="7"/>
     </row>
   </sheetData>
-  <sheetProtection password="9067" sheet="1" objects="1" scenarios="1"/>
+  <sheetProtection password="A892" sheet="1" objects="1" scenarios="1"/>
   <mergeCells count="1">
     <mergeCell ref="A4:E4"/>
   </mergeCells>
@@ -8793,7 +8793,7 @@
       <c r="A1005" s="7"/>
     </row>
   </sheetData>
-  <sheetProtection password="9643" sheet="1" objects="1" scenarios="1"/>
+  <sheetProtection password="E2BE" sheet="1" objects="1" scenarios="1"/>
   <mergeCells count="1">
     <mergeCell ref="A4:O4"/>
   </mergeCells>
@@ -11869,7 +11869,7 @@
       <c r="A1005" s="7"/>
     </row>
   </sheetData>
-  <sheetProtection password="AA59" sheet="1" objects="1" scenarios="1"/>
+  <sheetProtection password="C66B" sheet="1" objects="1" scenarios="1"/>
   <mergeCells count="1">
     <mergeCell ref="A4:D4"/>
   </mergeCells>
@@ -11988,7 +11988,7 @@
       <c r="H4" s="6"/>
     </row>
   </sheetData>
-  <sheetProtection password="A515" sheet="1" objects="1" scenarios="1"/>
+  <sheetProtection password="8AA9" sheet="1" objects="1" scenarios="1"/>
   <mergeCells count="1">
     <mergeCell ref="A4:H4"/>
   </mergeCells>
@@ -18143,7 +18143,7 @@
       <c r="D1005" s="7"/>
     </row>
   </sheetData>
-  <sheetProtection password="DF5B" sheet="1" objects="1" scenarios="1"/>
+  <sheetProtection password="A082" sheet="1" objects="1" scenarios="1"/>
   <mergeCells count="1">
     <mergeCell ref="A4:K4"/>
   </mergeCells>
@@ -22354,7 +22354,7 @@
       <c r="B1005" s="7"/>
     </row>
   </sheetData>
-  <sheetProtection password="F7A3" sheet="1" objects="1" scenarios="1"/>
+  <sheetProtection password="AE76" sheet="1" objects="1" scenarios="1"/>
   <mergeCells count="1">
     <mergeCell ref="A4:P4"/>
   </mergeCells>
@@ -28526,7 +28526,7 @@
       <c r="D1005" s="7"/>
     </row>
   </sheetData>
-  <sheetProtection password="ED24" sheet="1" objects="1" scenarios="1"/>
+  <sheetProtection password="F708" sheet="1" objects="1" scenarios="1"/>
   <mergeCells count="1">
     <mergeCell ref="A4:K4"/>
   </mergeCells>
@@ -28650,7 +28650,7 @@
       <c r="H4" s="6"/>
     </row>
   </sheetData>
-  <sheetProtection password="90C3" sheet="1" objects="1" scenarios="1"/>
+  <sheetProtection password="D6FC" sheet="1" objects="1" scenarios="1"/>
   <mergeCells count="1">
     <mergeCell ref="A4:H4"/>
   </mergeCells>
@@ -32436,7 +32436,7 @@
       <c r="A1005" s="7"/>
     </row>
   </sheetData>
-  <sheetProtection password="CF19" sheet="1" objects="1" scenarios="1"/>
+  <sheetProtection password="DBF1" sheet="1" objects="1" scenarios="1"/>
   <mergeCells count="1">
     <mergeCell ref="A4:H4"/>
   </mergeCells>
@@ -36526,7 +36526,7 @@
       <c r="B1005" s="7"/>
     </row>
   </sheetData>
-  <sheetProtection password="996A" sheet="1" objects="1" scenarios="1"/>
+  <sheetProtection password="A034" sheet="1" objects="1" scenarios="1"/>
   <mergeCells count="1">
     <mergeCell ref="A4:E4"/>
   </mergeCells>
@@ -40682,7 +40682,7 @@
       <c r="B1005" s="7"/>
     </row>
   </sheetData>
-  <sheetProtection password="F3FA" sheet="1" objects="1" scenarios="1"/>
+  <sheetProtection password="A666" sheet="1" objects="1" scenarios="1"/>
   <mergeCells count="1">
     <mergeCell ref="A4:K4"/>
   </mergeCells>
@@ -46878,7 +46878,7 @@
       <c r="D1005" s="7"/>
     </row>
   </sheetData>
-  <sheetProtection password="EF34" sheet="1" objects="1" scenarios="1"/>
+  <sheetProtection password="BFFB" sheet="1" objects="1" scenarios="1"/>
   <mergeCells count="1">
     <mergeCell ref="A4:N4"/>
   </mergeCells>
@@ -52249,7 +52249,7 @@
       <c r="C1005" s="7"/>
     </row>
   </sheetData>
-  <sheetProtection password="EAFE" sheet="1" objects="1" scenarios="1"/>
+  <sheetProtection password="FF1A" sheet="1" objects="1" scenarios="1"/>
   <mergeCells count="1">
     <mergeCell ref="A4:AD4"/>
   </mergeCells>
@@ -56469,7 +56469,7 @@
       <c r="B1005" s="7"/>
     </row>
   </sheetData>
-  <sheetProtection password="A4F0" sheet="1" objects="1" scenarios="1"/>
+  <sheetProtection password="DCB0" sheet="1" objects="1" scenarios="1"/>
   <mergeCells count="1">
     <mergeCell ref="A4:N4"/>
   </mergeCells>

</xml_diff>

<commit_message>
Updated single-information with additional enums to the 'library_strategy', 'library_selection' and 'library_source' fields
</commit_message>
<xml_diff>
--- a/dist/checklists/xlsx/dwc/single_cell_manifest_version_dwc_sc_rnaseq_v0.4.xlsx
+++ b/dist/checklists/xlsx/dwc/single_cell_manifest_version_dwc_sc_rnaseq_v0.4.xlsx
@@ -29,7 +29,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="824" uniqueCount="675">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="829" uniqueCount="680">
   <si>
     <t>key</t>
   </si>
@@ -835,6 +835,12 @@
     <t>Cdna</t>
   </si>
   <si>
+    <t>Cdna Oligo Dt</t>
+  </si>
+  <si>
+    <t>Cdna Randompriming</t>
+  </si>
+  <si>
     <t>Chip</t>
   </si>
   <si>
@@ -850,6 +856,9 @@
     <t>Hybrid Selection</t>
   </si>
   <si>
+    <t>Inverse Rrna</t>
+  </si>
+  <si>
     <t>Inverse Rrna Selection</t>
   </si>
   <si>
@@ -880,6 +889,9 @@
     <t>Pcr</t>
   </si>
   <si>
+    <t>Polya</t>
+  </si>
+  <si>
     <t>Race</t>
   </si>
   <si>
@@ -968,6 +980,9 @@
   </si>
   <si>
     <t>Ncrna-Seq</t>
+  </si>
+  <si>
+    <t>Nome-Seq</t>
   </si>
   <si>
     <t>Poolclone</t>
@@ -2505,7 +2520,7 @@
       </c>
     </row>
   </sheetData>
-  <sheetProtection password="B153" sheet="1" objects="1" scenarios="1"/>
+  <sheetProtection password="FED8" sheet="1" objects="1" scenarios="1"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
@@ -2527,16 +2542,16 @@
         <v>12</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>460</v>
+        <v>465</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>463</v>
+        <v>468</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>466</v>
+        <v>471</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>469</v>
+        <v>474</v>
       </c>
     </row>
     <row r="2" spans="1:5">
@@ -2544,16 +2559,16 @@
         <v>20</v>
       </c>
       <c r="B2" s="5" t="s">
-        <v>461</v>
+        <v>466</v>
       </c>
       <c r="C2" s="5" t="s">
-        <v>464</v>
+        <v>469</v>
       </c>
       <c r="D2" s="5" t="s">
-        <v>467</v>
+        <v>472</v>
       </c>
       <c r="E2" s="5" t="s">
-        <v>470</v>
+        <v>475</v>
       </c>
     </row>
     <row r="3" spans="1:5">
@@ -2561,16 +2576,16 @@
         <v>21</v>
       </c>
       <c r="B3" s="5" t="s">
-        <v>462</v>
+        <v>467</v>
       </c>
       <c r="C3" s="5" t="s">
-        <v>465</v>
+        <v>470</v>
       </c>
       <c r="D3" s="5" t="s">
-        <v>468</v>
+        <v>473</v>
       </c>
       <c r="E3" s="5" t="s">
-        <v>471</v>
+        <v>476</v>
       </c>
     </row>
     <row r="4" spans="1:5">
@@ -5586,7 +5601,7 @@
       <c r="A1005" s="7"/>
     </row>
   </sheetData>
-  <sheetProtection password="A892" sheet="1" objects="1" scenarios="1"/>
+  <sheetProtection password="971B" sheet="1" objects="1" scenarios="1"/>
   <mergeCells count="1">
     <mergeCell ref="A4:E4"/>
   </mergeCells>
@@ -5634,46 +5649,46 @@
         <v>12</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>486</v>
+        <v>491</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>489</v>
+        <v>494</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>492</v>
+        <v>497</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>495</v>
+        <v>500</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>498</v>
+        <v>503</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>501</v>
+        <v>506</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>504</v>
+        <v>509</v>
       </c>
       <c r="I1" s="1" t="s">
-        <v>507</v>
+        <v>512</v>
       </c>
       <c r="J1" s="1" t="s">
-        <v>510</v>
+        <v>515</v>
       </c>
       <c r="K1" s="1" t="s">
-        <v>513</v>
+        <v>518</v>
       </c>
       <c r="L1" s="1" t="s">
-        <v>516</v>
+        <v>521</v>
       </c>
       <c r="M1" s="1" t="s">
-        <v>519</v>
+        <v>524</v>
       </c>
       <c r="N1" s="1" t="s">
-        <v>522</v>
+        <v>527</v>
       </c>
       <c r="O1" s="1" t="s">
-        <v>524</v>
+        <v>529</v>
       </c>
     </row>
     <row r="2" spans="1:15">
@@ -5681,46 +5696,46 @@
         <v>20</v>
       </c>
       <c r="B2" s="5" t="s">
-        <v>487</v>
+        <v>492</v>
       </c>
       <c r="C2" s="5" t="s">
-        <v>490</v>
+        <v>495</v>
       </c>
       <c r="D2" s="5" t="s">
-        <v>493</v>
+        <v>498</v>
       </c>
       <c r="E2" s="5" t="s">
-        <v>496</v>
+        <v>501</v>
       </c>
       <c r="F2" s="5" t="s">
-        <v>499</v>
+        <v>504</v>
       </c>
       <c r="G2" s="5" t="s">
-        <v>502</v>
+        <v>507</v>
       </c>
       <c r="H2" s="5" t="s">
-        <v>505</v>
+        <v>510</v>
       </c>
       <c r="I2" s="5" t="s">
-        <v>508</v>
+        <v>513</v>
       </c>
       <c r="J2" s="5" t="s">
-        <v>511</v>
+        <v>516</v>
       </c>
       <c r="K2" s="5" t="s">
-        <v>514</v>
+        <v>519</v>
       </c>
       <c r="L2" s="5" t="s">
-        <v>517</v>
+        <v>522</v>
       </c>
       <c r="M2" s="5" t="s">
-        <v>520</v>
+        <v>525</v>
       </c>
       <c r="N2" s="5" t="s">
-        <v>508</v>
+        <v>513</v>
       </c>
       <c r="O2" s="5" t="s">
-        <v>525</v>
+        <v>530</v>
       </c>
     </row>
     <row r="3" spans="1:15">
@@ -5728,46 +5743,46 @@
         <v>21</v>
       </c>
       <c r="B3" s="5" t="s">
-        <v>488</v>
+        <v>493</v>
       </c>
       <c r="C3" s="5" t="s">
-        <v>491</v>
+        <v>496</v>
       </c>
       <c r="D3" s="5" t="s">
-        <v>494</v>
+        <v>499</v>
       </c>
       <c r="E3" s="5" t="s">
-        <v>497</v>
+        <v>502</v>
       </c>
       <c r="F3" s="5" t="s">
-        <v>500</v>
+        <v>505</v>
       </c>
       <c r="G3" s="5" t="s">
-        <v>503</v>
+        <v>508</v>
       </c>
       <c r="H3" s="5" t="s">
-        <v>506</v>
+        <v>511</v>
       </c>
       <c r="I3" s="5" t="s">
-        <v>509</v>
+        <v>514</v>
       </c>
       <c r="J3" s="5" t="s">
-        <v>512</v>
+        <v>517</v>
       </c>
       <c r="K3" s="5" t="s">
-        <v>515</v>
+        <v>520</v>
       </c>
       <c r="L3" s="5" t="s">
-        <v>518</v>
+        <v>523</v>
       </c>
       <c r="M3" s="5" t="s">
-        <v>521</v>
+        <v>526</v>
       </c>
       <c r="N3" s="5" t="s">
-        <v>523</v>
+        <v>528</v>
       </c>
       <c r="O3" s="5" t="s">
-        <v>526</v>
+        <v>531</v>
       </c>
     </row>
     <row r="4" spans="1:15">
@@ -8793,7 +8808,7 @@
       <c r="A1005" s="7"/>
     </row>
   </sheetData>
-  <sheetProtection password="E2BE" sheet="1" objects="1" scenarios="1"/>
+  <sheetProtection password="DB6D" sheet="1" objects="1" scenarios="1"/>
   <mergeCells count="1">
     <mergeCell ref="A4:O4"/>
   </mergeCells>
@@ -8820,13 +8835,13 @@
         <v>12</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>530</v>
+        <v>535</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>533</v>
+        <v>538</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>535</v>
+        <v>540</v>
       </c>
     </row>
     <row r="2" spans="1:4">
@@ -8834,13 +8849,13 @@
         <v>20</v>
       </c>
       <c r="B2" s="5" t="s">
-        <v>531</v>
+        <v>536</v>
       </c>
       <c r="C2" s="5" t="s">
-        <v>531</v>
+        <v>536</v>
       </c>
       <c r="D2" s="5" t="s">
-        <v>531</v>
+        <v>536</v>
       </c>
     </row>
     <row r="3" spans="1:4">
@@ -8848,13 +8863,13 @@
         <v>21</v>
       </c>
       <c r="B3" s="5" t="s">
-        <v>532</v>
+        <v>537</v>
       </c>
       <c r="C3" s="5" t="s">
-        <v>534</v>
+        <v>539</v>
       </c>
       <c r="D3" s="5" t="s">
-        <v>536</v>
+        <v>541</v>
       </c>
     </row>
     <row r="4" spans="1:4">
@@ -11869,7 +11884,7 @@
       <c r="A1005" s="7"/>
     </row>
   </sheetData>
-  <sheetProtection password="C66B" sheet="1" objects="1" scenarios="1"/>
+  <sheetProtection password="CD45" sheet="1" objects="1" scenarios="1"/>
   <mergeCells count="1">
     <mergeCell ref="A4:D4"/>
   </mergeCells>
@@ -11899,80 +11914,80 @@
   <sheetData>
     <row r="1" spans="1:8">
       <c r="A1" s="1" t="s">
-        <v>545</v>
+        <v>550</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>548</v>
+        <v>553</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>551</v>
+        <v>556</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>554</v>
+        <v>559</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>557</v>
+        <v>562</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>560</v>
+        <v>565</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>563</v>
+        <v>568</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>566</v>
+        <v>571</v>
       </c>
     </row>
     <row r="2" spans="1:8">
       <c r="A2" s="5" t="s">
-        <v>546</v>
+        <v>551</v>
       </c>
       <c r="B2" s="5" t="s">
-        <v>549</v>
+        <v>554</v>
       </c>
       <c r="C2" s="5" t="s">
-        <v>552</v>
+        <v>557</v>
       </c>
       <c r="D2" s="5" t="s">
-        <v>555</v>
+        <v>560</v>
       </c>
       <c r="E2" s="5" t="s">
-        <v>558</v>
+        <v>563</v>
       </c>
       <c r="F2" s="5" t="s">
-        <v>561</v>
+        <v>566</v>
       </c>
       <c r="G2" s="5" t="s">
-        <v>564</v>
+        <v>569</v>
       </c>
       <c r="H2" s="5" t="s">
-        <v>567</v>
+        <v>572</v>
       </c>
     </row>
     <row r="3" spans="1:8">
       <c r="A3" s="5" t="s">
-        <v>547</v>
+        <v>552</v>
       </c>
       <c r="B3" s="5" t="s">
-        <v>550</v>
+        <v>555</v>
       </c>
       <c r="C3" s="5" t="s">
-        <v>553</v>
+        <v>558</v>
       </c>
       <c r="D3" s="5" t="s">
-        <v>556</v>
+        <v>561</v>
       </c>
       <c r="E3" s="5" t="s">
-        <v>559</v>
+        <v>564</v>
       </c>
       <c r="F3" s="5" t="s">
-        <v>562</v>
+        <v>567</v>
       </c>
       <c r="G3" s="5" t="s">
-        <v>565</v>
+        <v>570</v>
       </c>
       <c r="H3" s="5" t="s">
-        <v>568</v>
+        <v>573</v>
       </c>
     </row>
     <row r="4" spans="1:8">
@@ -11988,7 +12003,7 @@
       <c r="H4" s="6"/>
     </row>
   </sheetData>
-  <sheetProtection password="8AA9" sheet="1" objects="1" scenarios="1"/>
+  <sheetProtection password="FF9A" sheet="1" objects="1" scenarios="1"/>
   <mergeCells count="1">
     <mergeCell ref="A4:H4"/>
   </mergeCells>
@@ -12021,34 +12036,34 @@
         <v>12</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>569</v>
+        <v>574</v>
       </c>
       <c r="C1" s="2" t="s">
         <v>165</v>
       </c>
       <c r="D1" s="2" t="s">
-        <v>330</v>
+        <v>335</v>
       </c>
       <c r="E1" s="2" t="s">
-        <v>570</v>
+        <v>575</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>580</v>
+        <v>585</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>583</v>
+        <v>588</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>586</v>
+        <v>591</v>
       </c>
       <c r="I1" s="2" t="s">
-        <v>574</v>
+        <v>579</v>
       </c>
       <c r="J1" s="1" t="s">
-        <v>591</v>
+        <v>596</v>
       </c>
       <c r="K1" s="1" t="s">
-        <v>594</v>
+        <v>599</v>
       </c>
     </row>
     <row r="2" spans="1:11">
@@ -12056,34 +12071,34 @@
         <v>20</v>
       </c>
       <c r="B2" s="5" t="s">
-        <v>577</v>
+        <v>582</v>
       </c>
       <c r="C2" s="5" t="s">
         <v>193</v>
       </c>
       <c r="D2" s="5" t="s">
-        <v>343</v>
+        <v>348</v>
       </c>
       <c r="E2" s="5" t="s">
-        <v>578</v>
+        <v>583</v>
       </c>
       <c r="F2" s="5" t="s">
-        <v>581</v>
+        <v>586</v>
       </c>
       <c r="G2" s="5" t="s">
-        <v>584</v>
+        <v>589</v>
       </c>
       <c r="H2" s="5" t="s">
-        <v>587</v>
+        <v>592</v>
       </c>
       <c r="I2" s="5" t="s">
-        <v>589</v>
+        <v>594</v>
       </c>
       <c r="J2" s="5" t="s">
-        <v>592</v>
+        <v>597</v>
       </c>
       <c r="K2" s="5" t="s">
-        <v>595</v>
+        <v>600</v>
       </c>
     </row>
     <row r="3" spans="1:11">
@@ -12097,28 +12112,28 @@
         <v>194</v>
       </c>
       <c r="D3" s="5" t="s">
-        <v>344</v>
+        <v>349</v>
       </c>
       <c r="E3" s="5" t="s">
-        <v>579</v>
+        <v>584</v>
       </c>
       <c r="F3" s="5" t="s">
-        <v>582</v>
+        <v>587</v>
       </c>
       <c r="G3" s="5" t="s">
-        <v>585</v>
+        <v>590</v>
       </c>
       <c r="H3" s="5" t="s">
-        <v>588</v>
+        <v>593</v>
       </c>
       <c r="I3" s="5" t="s">
-        <v>590</v>
+        <v>595</v>
       </c>
       <c r="J3" s="5" t="s">
-        <v>593</v>
+        <v>598</v>
       </c>
       <c r="K3" s="5" t="s">
-        <v>596</v>
+        <v>601</v>
       </c>
     </row>
     <row r="4" spans="1:11">
@@ -18143,7 +18158,7 @@
       <c r="D1005" s="7"/>
     </row>
   </sheetData>
-  <sheetProtection password="A082" sheet="1" objects="1" scenarios="1"/>
+  <sheetProtection password="F7C1" sheet="1" objects="1" scenarios="1"/>
   <mergeCells count="1">
     <mergeCell ref="A4:K4"/>
   </mergeCells>
@@ -18184,49 +18199,49 @@
         <v>12</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>597</v>
+        <v>602</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>613</v>
+        <v>618</v>
       </c>
       <c r="D1" s="2" t="s">
-        <v>472</v>
+        <v>477</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>617</v>
+        <v>622</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>620</v>
+        <v>625</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>623</v>
+        <v>628</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>626</v>
+        <v>631</v>
       </c>
       <c r="I1" s="1" t="s">
-        <v>629</v>
+        <v>634</v>
       </c>
       <c r="J1" s="1" t="s">
-        <v>632</v>
+        <v>637</v>
       </c>
       <c r="K1" s="1" t="s">
-        <v>634</v>
+        <v>639</v>
       </c>
       <c r="L1" s="1" t="s">
-        <v>637</v>
+        <v>642</v>
       </c>
       <c r="M1" s="1" t="s">
-        <v>640</v>
+        <v>645</v>
       </c>
       <c r="N1" s="1" t="s">
-        <v>642</v>
+        <v>647</v>
       </c>
       <c r="O1" s="1" t="s">
-        <v>644</v>
+        <v>649</v>
       </c>
       <c r="P1" s="1" t="s">
-        <v>646</v>
+        <v>651</v>
       </c>
     </row>
     <row r="2" spans="1:16">
@@ -18234,49 +18249,49 @@
         <v>20</v>
       </c>
       <c r="B2" s="5" t="s">
-        <v>611</v>
+        <v>616</v>
       </c>
       <c r="C2" s="5" t="s">
-        <v>598</v>
+        <v>603</v>
       </c>
       <c r="D2" s="5" t="s">
-        <v>615</v>
+        <v>620</v>
       </c>
       <c r="E2" s="5" t="s">
-        <v>618</v>
+        <v>623</v>
       </c>
       <c r="F2" s="5" t="s">
-        <v>621</v>
+        <v>626</v>
       </c>
       <c r="G2" s="5" t="s">
-        <v>624</v>
+        <v>629</v>
       </c>
       <c r="H2" s="5" t="s">
-        <v>627</v>
+        <v>632</v>
       </c>
       <c r="I2" s="5" t="s">
-        <v>630</v>
+        <v>635</v>
       </c>
       <c r="J2" s="5" t="s">
-        <v>633</v>
+        <v>638</v>
       </c>
       <c r="K2" s="5" t="s">
-        <v>635</v>
+        <v>640</v>
       </c>
       <c r="L2" s="5" t="s">
-        <v>638</v>
+        <v>643</v>
       </c>
       <c r="M2" s="5" t="s">
-        <v>641</v>
+        <v>646</v>
       </c>
       <c r="N2" s="5" t="s">
-        <v>643</v>
+        <v>648</v>
       </c>
       <c r="O2" s="5" t="s">
-        <v>645</v>
+        <v>650</v>
       </c>
       <c r="P2" s="5" t="s">
-        <v>647</v>
+        <v>652</v>
       </c>
     </row>
     <row r="3" spans="1:16">
@@ -18284,37 +18299,37 @@
         <v>21</v>
       </c>
       <c r="B3" s="5" t="s">
-        <v>612</v>
+        <v>617</v>
       </c>
       <c r="C3" s="5" t="s">
-        <v>614</v>
+        <v>619</v>
       </c>
       <c r="D3" s="5" t="s">
-        <v>616</v>
+        <v>621</v>
       </c>
       <c r="E3" s="5" t="s">
-        <v>619</v>
+        <v>624</v>
       </c>
       <c r="F3" s="5" t="s">
-        <v>622</v>
+        <v>627</v>
       </c>
       <c r="G3" s="5" t="s">
-        <v>625</v>
+        <v>630</v>
       </c>
       <c r="H3" s="5" t="s">
-        <v>628</v>
+        <v>633</v>
       </c>
       <c r="I3" s="5" t="s">
-        <v>631</v>
+        <v>636</v>
       </c>
       <c r="J3" s="5" t="s">
         <v>258</v>
       </c>
       <c r="K3" s="5" t="s">
-        <v>636</v>
+        <v>641</v>
       </c>
       <c r="L3" s="5" t="s">
-        <v>639</v>
+        <v>644</v>
       </c>
       <c r="M3" s="5" t="s">
         <v>258</v>
@@ -22354,7 +22369,7 @@
       <c r="B1005" s="7"/>
     </row>
   </sheetData>
-  <sheetProtection password="AE76" sheet="1" objects="1" scenarios="1"/>
+  <sheetProtection password="AF3D" sheet="1" objects="1" scenarios="1"/>
   <mergeCells count="1">
     <mergeCell ref="A4:P4"/>
   </mergeCells>
@@ -22404,34 +22419,34 @@
         <v>12</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>569</v>
+        <v>574</v>
       </c>
       <c r="C1" s="2" t="s">
         <v>165</v>
       </c>
       <c r="D1" s="2" t="s">
-        <v>597</v>
+        <v>602</v>
       </c>
       <c r="E1" s="2" t="s">
-        <v>648</v>
+        <v>653</v>
       </c>
       <c r="F1" s="2" t="s">
-        <v>649</v>
+        <v>654</v>
       </c>
       <c r="G1" s="2" t="s">
-        <v>650</v>
+        <v>655</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>664</v>
+        <v>669</v>
       </c>
       <c r="I1" s="1" t="s">
-        <v>667</v>
+        <v>672</v>
       </c>
       <c r="J1" s="1" t="s">
-        <v>670</v>
+        <v>675</v>
       </c>
       <c r="K1" s="1" t="s">
-        <v>673</v>
+        <v>678</v>
       </c>
     </row>
     <row r="2" spans="1:11">
@@ -22439,34 +22454,34 @@
         <v>20</v>
       </c>
       <c r="B2" s="5" t="s">
-        <v>655</v>
+        <v>660</v>
       </c>
       <c r="C2" s="5" t="s">
-        <v>657</v>
+        <v>662</v>
       </c>
       <c r="D2" s="5" t="s">
-        <v>611</v>
+        <v>616</v>
       </c>
       <c r="E2" s="5" t="s">
-        <v>658</v>
+        <v>663</v>
       </c>
       <c r="F2" s="5" t="s">
-        <v>660</v>
+        <v>665</v>
       </c>
       <c r="G2" s="5" t="s">
-        <v>662</v>
+        <v>667</v>
       </c>
       <c r="H2" s="5" t="s">
-        <v>665</v>
+        <v>670</v>
       </c>
       <c r="I2" s="5" t="s">
-        <v>668</v>
+        <v>673</v>
       </c>
       <c r="J2" s="5" t="s">
-        <v>671</v>
+        <v>676</v>
       </c>
       <c r="K2" s="5" t="s">
-        <v>674</v>
+        <v>679</v>
       </c>
     </row>
     <row r="3" spans="1:11">
@@ -22474,31 +22489,31 @@
         <v>21</v>
       </c>
       <c r="B3" s="5" t="s">
-        <v>656</v>
+        <v>661</v>
       </c>
       <c r="C3" s="5" t="s">
         <v>194</v>
       </c>
       <c r="D3" s="5" t="s">
-        <v>612</v>
+        <v>617</v>
       </c>
       <c r="E3" s="5" t="s">
-        <v>659</v>
+        <v>664</v>
       </c>
       <c r="F3" s="5" t="s">
-        <v>661</v>
+        <v>666</v>
       </c>
       <c r="G3" s="5" t="s">
-        <v>663</v>
+        <v>668</v>
       </c>
       <c r="H3" s="5" t="s">
-        <v>666</v>
+        <v>671</v>
       </c>
       <c r="I3" s="5" t="s">
-        <v>669</v>
+        <v>674</v>
       </c>
       <c r="J3" s="5" t="s">
-        <v>672</v>
+        <v>677</v>
       </c>
       <c r="K3" s="5" t="s">
         <v>29</v>
@@ -28526,7 +28541,7 @@
       <c r="D1005" s="7"/>
     </row>
   </sheetData>
-  <sheetProtection password="F708" sheet="1" objects="1" scenarios="1"/>
+  <sheetProtection password="BBD1" sheet="1" objects="1" scenarios="1"/>
   <mergeCells count="1">
     <mergeCell ref="A4:K4"/>
   </mergeCells>
@@ -28650,7 +28665,7 @@
       <c r="H4" s="6"/>
     </row>
   </sheetData>
-  <sheetProtection password="D6FC" sheet="1" objects="1" scenarios="1"/>
+  <sheetProtection password="82C8" sheet="1" objects="1" scenarios="1"/>
   <mergeCells count="1">
     <mergeCell ref="A4:H4"/>
   </mergeCells>
@@ -28684,12 +28699,12 @@
   <sheetData>
     <row r="5" spans="4:30">
       <c r="D5" t="s">
-        <v>373</v>
+        <v>378</v>
       </c>
     </row>
     <row r="6" spans="4:30">
       <c r="D6" t="s">
-        <v>374</v>
+        <v>379</v>
       </c>
       <c r="F6" t="s">
         <v>39</v>
@@ -28698,12 +28713,12 @@
         <v>265</v>
       </c>
       <c r="AD6" t="s">
-        <v>292</v>
+        <v>296</v>
       </c>
     </row>
     <row r="7" spans="4:30">
       <c r="D7" t="s">
-        <v>375</v>
+        <v>380</v>
       </c>
       <c r="F7" t="s">
         <v>40</v>
@@ -28712,12 +28727,12 @@
         <v>266</v>
       </c>
       <c r="AD7" t="s">
-        <v>293</v>
+        <v>297</v>
       </c>
     </row>
     <row r="8" spans="4:30">
       <c r="D8" t="s">
-        <v>376</v>
+        <v>381</v>
       </c>
       <c r="F8" t="s">
         <v>41</v>
@@ -28726,12 +28741,12 @@
         <v>267</v>
       </c>
       <c r="AD8" t="s">
-        <v>294</v>
+        <v>298</v>
       </c>
     </row>
     <row r="9" spans="4:30">
       <c r="D9" t="s">
-        <v>377</v>
+        <v>382</v>
       </c>
       <c r="F9" t="s">
         <v>42</v>
@@ -28740,12 +28755,12 @@
         <v>268</v>
       </c>
       <c r="AD9" t="s">
-        <v>295</v>
+        <v>299</v>
       </c>
     </row>
     <row r="10" spans="4:30">
       <c r="D10" t="s">
-        <v>378</v>
+        <v>383</v>
       </c>
       <c r="F10" t="s">
         <v>43</v>
@@ -28754,12 +28769,12 @@
         <v>269</v>
       </c>
       <c r="AD10" t="s">
-        <v>269</v>
+        <v>271</v>
       </c>
     </row>
     <row r="11" spans="4:30">
       <c r="D11" t="s">
-        <v>379</v>
+        <v>384</v>
       </c>
       <c r="F11" t="s">
         <v>44</v>
@@ -28768,12 +28783,12 @@
         <v>270</v>
       </c>
       <c r="AD11" t="s">
-        <v>296</v>
+        <v>300</v>
       </c>
     </row>
     <row r="12" spans="4:30">
       <c r="D12" t="s">
-        <v>380</v>
+        <v>385</v>
       </c>
       <c r="F12" t="s">
         <v>45</v>
@@ -28782,12 +28797,12 @@
         <v>271</v>
       </c>
       <c r="AD12" t="s">
-        <v>297</v>
+        <v>301</v>
       </c>
     </row>
     <row r="13" spans="4:30">
       <c r="D13" t="s">
-        <v>381</v>
+        <v>386</v>
       </c>
       <c r="F13" t="s">
         <v>46</v>
@@ -28796,530 +28811,545 @@
         <v>272</v>
       </c>
       <c r="AD13" t="s">
-        <v>298</v>
+        <v>302</v>
       </c>
     </row>
     <row r="14" spans="4:30">
       <c r="D14" t="s">
-        <v>382</v>
+        <v>387</v>
       </c>
       <c r="AB14" t="s">
         <v>273</v>
       </c>
       <c r="AD14" t="s">
-        <v>299</v>
+        <v>303</v>
       </c>
     </row>
     <row r="15" spans="4:30">
       <c r="D15" t="s">
-        <v>383</v>
+        <v>388</v>
       </c>
       <c r="AB15" t="s">
         <v>274</v>
       </c>
       <c r="AD15" t="s">
-        <v>300</v>
+        <v>304</v>
       </c>
     </row>
     <row r="16" spans="4:30">
       <c r="D16" t="s">
-        <v>384</v>
+        <v>389</v>
       </c>
       <c r="AB16" t="s">
         <v>275</v>
       </c>
       <c r="AD16" t="s">
-        <v>301</v>
+        <v>305</v>
       </c>
     </row>
     <row r="17" spans="4:30">
       <c r="D17" t="s">
-        <v>385</v>
+        <v>390</v>
       </c>
       <c r="AB17" t="s">
         <v>276</v>
       </c>
       <c r="AD17" t="s">
-        <v>302</v>
+        <v>306</v>
       </c>
     </row>
     <row r="18" spans="4:30">
       <c r="D18" t="s">
-        <v>386</v>
+        <v>391</v>
       </c>
       <c r="AB18" t="s">
         <v>277</v>
       </c>
       <c r="AD18" t="s">
-        <v>303</v>
+        <v>307</v>
       </c>
     </row>
     <row r="19" spans="4:30">
       <c r="D19" t="s">
-        <v>387</v>
+        <v>392</v>
       </c>
       <c r="AB19" t="s">
         <v>278</v>
       </c>
       <c r="AD19" t="s">
-        <v>304</v>
+        <v>308</v>
       </c>
     </row>
     <row r="20" spans="4:30">
       <c r="D20" t="s">
-        <v>388</v>
+        <v>393</v>
       </c>
       <c r="AB20" t="s">
         <v>279</v>
       </c>
       <c r="AD20" t="s">
-        <v>305</v>
+        <v>309</v>
       </c>
     </row>
     <row r="21" spans="4:30">
       <c r="D21" t="s">
-        <v>389</v>
+        <v>394</v>
       </c>
       <c r="AB21" t="s">
         <v>280</v>
       </c>
       <c r="AD21" t="s">
-        <v>306</v>
+        <v>310</v>
       </c>
     </row>
     <row r="22" spans="4:30">
       <c r="D22" t="s">
-        <v>390</v>
+        <v>395</v>
       </c>
       <c r="AB22" t="s">
         <v>281</v>
       </c>
       <c r="AD22" t="s">
-        <v>307</v>
+        <v>311</v>
       </c>
     </row>
     <row r="23" spans="4:30">
       <c r="D23" t="s">
-        <v>391</v>
+        <v>396</v>
       </c>
       <c r="AB23" t="s">
         <v>282</v>
       </c>
       <c r="AD23" t="s">
-        <v>308</v>
+        <v>312</v>
       </c>
     </row>
     <row r="24" spans="4:30">
       <c r="D24" t="s">
-        <v>392</v>
+        <v>397</v>
       </c>
       <c r="AB24" t="s">
         <v>283</v>
       </c>
       <c r="AD24" t="s">
-        <v>309</v>
+        <v>313</v>
       </c>
     </row>
     <row r="25" spans="4:30">
       <c r="D25" t="s">
-        <v>393</v>
+        <v>398</v>
       </c>
       <c r="AB25" t="s">
         <v>284</v>
       </c>
       <c r="AD25" t="s">
-        <v>310</v>
+        <v>314</v>
       </c>
     </row>
     <row r="26" spans="4:30">
       <c r="D26" t="s">
-        <v>394</v>
+        <v>399</v>
       </c>
       <c r="AB26" t="s">
         <v>285</v>
       </c>
       <c r="AD26" t="s">
-        <v>311</v>
+        <v>315</v>
       </c>
     </row>
     <row r="27" spans="4:30">
       <c r="D27" t="s">
-        <v>395</v>
+        <v>400</v>
       </c>
       <c r="AB27" t="s">
         <v>286</v>
       </c>
       <c r="AD27" t="s">
-        <v>312</v>
+        <v>316</v>
       </c>
     </row>
     <row r="28" spans="4:30">
       <c r="D28" t="s">
-        <v>396</v>
+        <v>401</v>
       </c>
       <c r="AB28" t="s">
         <v>287</v>
       </c>
       <c r="AD28" t="s">
-        <v>280</v>
+        <v>317</v>
       </c>
     </row>
     <row r="29" spans="4:30">
       <c r="D29" t="s">
-        <v>397</v>
+        <v>402</v>
       </c>
       <c r="AB29" t="s">
         <v>288</v>
       </c>
       <c r="AD29" t="s">
-        <v>313</v>
+        <v>283</v>
       </c>
     </row>
     <row r="30" spans="4:30">
       <c r="D30" t="s">
-        <v>398</v>
+        <v>403</v>
       </c>
       <c r="AB30" t="s">
         <v>289</v>
       </c>
       <c r="AD30" t="s">
-        <v>314</v>
+        <v>318</v>
       </c>
     </row>
     <row r="31" spans="4:30">
       <c r="D31" t="s">
-        <v>399</v>
+        <v>404</v>
       </c>
       <c r="AB31" t="s">
         <v>290</v>
       </c>
       <c r="AD31" t="s">
-        <v>315</v>
+        <v>319</v>
       </c>
     </row>
     <row r="32" spans="4:30">
       <c r="D32" t="s">
-        <v>400</v>
+        <v>405</v>
       </c>
       <c r="AB32" t="s">
         <v>291</v>
       </c>
       <c r="AD32" t="s">
-        <v>316</v>
+        <v>320</v>
       </c>
     </row>
     <row r="33" spans="4:30">
       <c r="D33" t="s">
-        <v>401</v>
+        <v>406</v>
+      </c>
+      <c r="AB33" t="s">
+        <v>292</v>
       </c>
       <c r="AD33" t="s">
-        <v>317</v>
+        <v>321</v>
       </c>
     </row>
     <row r="34" spans="4:30">
       <c r="D34" t="s">
-        <v>402</v>
+        <v>407</v>
+      </c>
+      <c r="AB34" t="s">
+        <v>293</v>
       </c>
       <c r="AD34" t="s">
-        <v>318</v>
+        <v>322</v>
       </c>
     </row>
     <row r="35" spans="4:30">
       <c r="D35" t="s">
-        <v>403</v>
+        <v>408</v>
+      </c>
+      <c r="AB35" t="s">
+        <v>294</v>
       </c>
       <c r="AD35" t="s">
-        <v>319</v>
+        <v>323</v>
       </c>
     </row>
     <row r="36" spans="4:30">
       <c r="D36" t="s">
-        <v>404</v>
+        <v>409</v>
+      </c>
+      <c r="AB36" t="s">
+        <v>295</v>
       </c>
       <c r="AD36" t="s">
-        <v>320</v>
+        <v>324</v>
       </c>
     </row>
     <row r="37" spans="4:30">
       <c r="D37" t="s">
-        <v>405</v>
+        <v>410</v>
       </c>
       <c r="AD37" t="s">
-        <v>321</v>
+        <v>325</v>
       </c>
     </row>
     <row r="38" spans="4:30">
       <c r="D38" t="s">
-        <v>406</v>
+        <v>411</v>
       </c>
       <c r="AD38" t="s">
-        <v>322</v>
+        <v>326</v>
       </c>
     </row>
     <row r="39" spans="4:30">
       <c r="D39" t="s">
-        <v>407</v>
+        <v>412</v>
       </c>
       <c r="AD39" t="s">
-        <v>323</v>
+        <v>327</v>
       </c>
     </row>
     <row r="40" spans="4:30">
       <c r="D40" t="s">
-        <v>408</v>
+        <v>413</v>
       </c>
       <c r="AD40" t="s">
-        <v>324</v>
+        <v>328</v>
       </c>
     </row>
     <row r="41" spans="4:30">
       <c r="D41" t="s">
-        <v>409</v>
+        <v>414</v>
       </c>
       <c r="AD41" t="s">
-        <v>325</v>
+        <v>329</v>
       </c>
     </row>
     <row r="42" spans="4:30">
       <c r="D42" t="s">
-        <v>410</v>
+        <v>415</v>
       </c>
       <c r="AD42" t="s">
-        <v>326</v>
+        <v>330</v>
       </c>
     </row>
     <row r="43" spans="4:30">
       <c r="D43" t="s">
-        <v>411</v>
+        <v>416</v>
       </c>
       <c r="AD43" t="s">
-        <v>327</v>
+        <v>331</v>
       </c>
     </row>
     <row r="44" spans="4:30">
       <c r="D44" t="s">
-        <v>412</v>
+        <v>417</v>
       </c>
       <c r="AD44" t="s">
-        <v>328</v>
+        <v>332</v>
       </c>
     </row>
     <row r="45" spans="4:30">
       <c r="D45" t="s">
-        <v>413</v>
+        <v>418</v>
       </c>
       <c r="AD45" t="s">
-        <v>329</v>
+        <v>333</v>
       </c>
     </row>
     <row r="46" spans="4:30">
       <c r="D46" t="s">
-        <v>414</v>
+        <v>419</v>
+      </c>
+      <c r="AD46" t="s">
+        <v>334</v>
       </c>
     </row>
     <row r="47" spans="4:30">
       <c r="D47" t="s">
-        <v>415</v>
+        <v>420</v>
       </c>
     </row>
     <row r="48" spans="4:30">
       <c r="D48" t="s">
-        <v>416</v>
+        <v>421</v>
       </c>
     </row>
     <row r="49" spans="4:4">
       <c r="D49" t="s">
-        <v>417</v>
+        <v>422</v>
       </c>
     </row>
     <row r="50" spans="4:4">
       <c r="D50" t="s">
-        <v>418</v>
+        <v>423</v>
       </c>
     </row>
     <row r="51" spans="4:4">
       <c r="D51" t="s">
-        <v>419</v>
+        <v>424</v>
       </c>
     </row>
     <row r="52" spans="4:4">
       <c r="D52" t="s">
-        <v>420</v>
+        <v>425</v>
       </c>
     </row>
     <row r="53" spans="4:4">
       <c r="D53" t="s">
-        <v>421</v>
+        <v>426</v>
       </c>
     </row>
     <row r="54" spans="4:4">
       <c r="D54" t="s">
-        <v>422</v>
+        <v>427</v>
       </c>
     </row>
     <row r="55" spans="4:4">
       <c r="D55" t="s">
-        <v>423</v>
+        <v>428</v>
       </c>
     </row>
     <row r="56" spans="4:4">
       <c r="D56" t="s">
-        <v>424</v>
+        <v>429</v>
       </c>
     </row>
     <row r="57" spans="4:4">
       <c r="D57" t="s">
-        <v>425</v>
+        <v>430</v>
       </c>
     </row>
     <row r="58" spans="4:4">
       <c r="D58" t="s">
-        <v>426</v>
+        <v>431</v>
       </c>
     </row>
     <row r="59" spans="4:4">
       <c r="D59" t="s">
-        <v>427</v>
+        <v>432</v>
       </c>
     </row>
     <row r="60" spans="4:4">
       <c r="D60" t="s">
-        <v>428</v>
+        <v>433</v>
       </c>
     </row>
     <row r="61" spans="4:4">
       <c r="D61" t="s">
-        <v>429</v>
+        <v>434</v>
       </c>
     </row>
     <row r="62" spans="4:4">
       <c r="D62" t="s">
-        <v>430</v>
+        <v>435</v>
       </c>
     </row>
     <row r="63" spans="4:4">
       <c r="D63" t="s">
-        <v>431</v>
+        <v>436</v>
       </c>
     </row>
     <row r="64" spans="4:4">
       <c r="D64" t="s">
-        <v>432</v>
+        <v>437</v>
       </c>
     </row>
     <row r="65" spans="4:4">
       <c r="D65" t="s">
-        <v>433</v>
+        <v>438</v>
       </c>
     </row>
     <row r="66" spans="4:4">
       <c r="D66" t="s">
-        <v>434</v>
+        <v>439</v>
       </c>
     </row>
     <row r="67" spans="4:4">
       <c r="D67" t="s">
-        <v>435</v>
+        <v>440</v>
       </c>
     </row>
     <row r="68" spans="4:4">
       <c r="D68" t="s">
-        <v>436</v>
+        <v>441</v>
       </c>
     </row>
     <row r="69" spans="4:4">
       <c r="D69" t="s">
-        <v>437</v>
+        <v>442</v>
       </c>
     </row>
     <row r="70" spans="4:4">
       <c r="D70" t="s">
-        <v>438</v>
+        <v>443</v>
       </c>
     </row>
     <row r="71" spans="4:4">
       <c r="D71" t="s">
-        <v>439</v>
+        <v>444</v>
       </c>
     </row>
     <row r="72" spans="4:4">
       <c r="D72" t="s">
-        <v>440</v>
+        <v>445</v>
       </c>
     </row>
     <row r="73" spans="4:4">
       <c r="D73" t="s">
-        <v>441</v>
+        <v>446</v>
       </c>
     </row>
     <row r="74" spans="4:4">
       <c r="D74" t="s">
-        <v>442</v>
+        <v>447</v>
       </c>
     </row>
     <row r="75" spans="4:4">
       <c r="D75" t="s">
-        <v>443</v>
+        <v>448</v>
       </c>
     </row>
     <row r="76" spans="4:4">
       <c r="D76" t="s">
-        <v>444</v>
+        <v>449</v>
       </c>
     </row>
     <row r="77" spans="4:4">
       <c r="D77" t="s">
-        <v>445</v>
+        <v>450</v>
       </c>
     </row>
     <row r="78" spans="4:4">
       <c r="D78" t="s">
-        <v>446</v>
+        <v>451</v>
       </c>
     </row>
     <row r="79" spans="4:4">
       <c r="D79" t="s">
-        <v>447</v>
+        <v>452</v>
       </c>
     </row>
     <row r="80" spans="4:4">
       <c r="D80" t="s">
-        <v>448</v>
+        <v>453</v>
       </c>
     </row>
     <row r="81" spans="4:4">
       <c r="D81" t="s">
-        <v>449</v>
+        <v>454</v>
       </c>
     </row>
     <row r="82" spans="4:4">
       <c r="D82" t="s">
-        <v>450</v>
+        <v>455</v>
       </c>
     </row>
     <row r="83" spans="4:4">
       <c r="D83" t="s">
-        <v>451</v>
+        <v>456</v>
       </c>
     </row>
     <row r="84" spans="4:4">
       <c r="D84" t="s">
-        <v>452</v>
+        <v>457</v>
       </c>
     </row>
     <row r="85" spans="4:4">
       <c r="D85" t="s">
-        <v>453</v>
+        <v>458</v>
       </c>
     </row>
     <row r="86" spans="4:4">
       <c r="D86" t="s">
-        <v>454</v>
+        <v>459</v>
       </c>
     </row>
     <row r="87" spans="4:4">
       <c r="D87" t="s">
-        <v>455</v>
+        <v>460</v>
       </c>
     </row>
   </sheetData>
@@ -32436,7 +32466,7 @@
       <c r="A1005" s="7"/>
     </row>
   </sheetData>
-  <sheetProtection password="DBF1" sheet="1" objects="1" scenarios="1"/>
+  <sheetProtection password="8C47" sheet="1" objects="1" scenarios="1"/>
   <mergeCells count="1">
     <mergeCell ref="A4:H4"/>
   </mergeCells>
@@ -36526,7 +36556,7 @@
       <c r="B1005" s="7"/>
     </row>
   </sheetData>
-  <sheetProtection password="A034" sheet="1" objects="1" scenarios="1"/>
+  <sheetProtection password="D8D6" sheet="1" objects="1" scenarios="1"/>
   <mergeCells count="1">
     <mergeCell ref="A4:E4"/>
   </mergeCells>
@@ -40682,7 +40712,7 @@
       <c r="B1005" s="7"/>
     </row>
   </sheetData>
-  <sheetProtection password="A666" sheet="1" objects="1" scenarios="1"/>
+  <sheetProtection password="92BB" sheet="1" objects="1" scenarios="1"/>
   <mergeCells count="1">
     <mergeCell ref="A4:K4"/>
   </mergeCells>
@@ -46878,7 +46908,7 @@
       <c r="D1005" s="7"/>
     </row>
   </sheetData>
-  <sheetProtection password="BFFB" sheet="1" objects="1" scenarios="1"/>
+  <sheetProtection password="E1A5" sheet="1" objects="1" scenarios="1"/>
   <mergeCells count="1">
     <mergeCell ref="A4:N4"/>
   </mergeCells>
@@ -52249,7 +52279,7 @@
       <c r="C1005" s="7"/>
     </row>
   </sheetData>
-  <sheetProtection password="FF1A" sheet="1" objects="1" scenarios="1"/>
+  <sheetProtection password="C639" sheet="1" objects="1" scenarios="1"/>
   <mergeCells count="1">
     <mergeCell ref="A4:AD4"/>
   </mergeCells>
@@ -52281,13 +52311,13 @@
       <formula1>",Cd41+,Cd41-"</formula1>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" prompt="Choose from the list" sqref="AB5:AB1005">
-      <formula1>HiddenDropdowns!$AB$5:$AB$32</formula1>
+      <formula1>HiddenDropdowns!$AB$5:$AB$36</formula1>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" prompt="Choose from the list" sqref="AC5:AC1005">
-      <formula1>",Genomic,Metagenomic,Metatranscriptomic,Other,Synthetic,Transcriptomic,Viral Rna"</formula1>
+      <formula1>",Genomic,Genomic Single Cell,Metagenomic,Metatranscriptomic,Other,Synthetic,Transcriptomic,Transcriptomic Single Cell,Viral Rna"</formula1>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" prompt="Choose from the list" sqref="AD5:AD1005">
-      <formula1>HiddenDropdowns!$AD$5:$AD$45</formula1>
+      <formula1>HiddenDropdowns!$AD$5:$AD$46</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -52319,43 +52349,43 @@
         <v>12</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>330</v>
+        <v>335</v>
       </c>
       <c r="C1" s="2" t="s">
-        <v>331</v>
+        <v>336</v>
       </c>
       <c r="D1" s="2" t="s">
-        <v>332</v>
+        <v>337</v>
       </c>
       <c r="E1" s="2" t="s">
-        <v>333</v>
+        <v>338</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>351</v>
+        <v>356</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>354</v>
+        <v>359</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>357</v>
+        <v>362</v>
       </c>
       <c r="I1" s="1" t="s">
-        <v>359</v>
+        <v>364</v>
       </c>
       <c r="J1" s="1" t="s">
-        <v>362</v>
+        <v>367</v>
       </c>
       <c r="K1" s="1" t="s">
-        <v>364</v>
+        <v>369</v>
       </c>
       <c r="L1" s="2" t="s">
-        <v>340</v>
+        <v>345</v>
       </c>
       <c r="M1" s="1" t="s">
-        <v>367</v>
+        <v>372</v>
       </c>
       <c r="N1" s="1" t="s">
-        <v>370</v>
+        <v>375</v>
       </c>
     </row>
     <row r="2" spans="1:14">
@@ -52363,43 +52393,43 @@
         <v>20</v>
       </c>
       <c r="B2" s="5" t="s">
-        <v>343</v>
+        <v>348</v>
       </c>
       <c r="C2" s="5" t="s">
-        <v>345</v>
+        <v>350</v>
       </c>
       <c r="D2" s="5" t="s">
-        <v>347</v>
+        <v>352</v>
       </c>
       <c r="E2" s="5" t="s">
-        <v>349</v>
+        <v>354</v>
       </c>
       <c r="F2" s="5" t="s">
-        <v>352</v>
+        <v>357</v>
       </c>
       <c r="G2" s="5" t="s">
-        <v>355</v>
+        <v>360</v>
       </c>
       <c r="H2" s="5" t="s">
-        <v>358</v>
+        <v>363</v>
       </c>
       <c r="I2" s="5" t="s">
-        <v>360</v>
+        <v>365</v>
       </c>
       <c r="J2" s="5" t="s">
-        <v>363</v>
+        <v>368</v>
       </c>
       <c r="K2" s="5" t="s">
-        <v>363</v>
+        <v>368</v>
       </c>
       <c r="L2" s="5" t="s">
-        <v>365</v>
+        <v>370</v>
       </c>
       <c r="M2" s="5" t="s">
-        <v>368</v>
+        <v>373</v>
       </c>
       <c r="N2" s="5" t="s">
-        <v>371</v>
+        <v>376</v>
       </c>
     </row>
     <row r="3" spans="1:14">
@@ -52407,43 +52437,43 @@
         <v>21</v>
       </c>
       <c r="B3" s="5" t="s">
-        <v>344</v>
+        <v>349</v>
       </c>
       <c r="C3" s="5" t="s">
-        <v>346</v>
+        <v>351</v>
       </c>
       <c r="D3" s="5" t="s">
-        <v>348</v>
+        <v>353</v>
       </c>
       <c r="E3" s="5" t="s">
-        <v>350</v>
+        <v>355</v>
       </c>
       <c r="F3" s="5" t="s">
-        <v>353</v>
+        <v>358</v>
       </c>
       <c r="G3" s="5" t="s">
-        <v>356</v>
+        <v>361</v>
       </c>
       <c r="H3" s="5" t="s">
         <v>150</v>
       </c>
       <c r="I3" s="5" t="s">
-        <v>361</v>
+        <v>366</v>
       </c>
       <c r="J3" s="5" t="s">
         <v>150</v>
       </c>
       <c r="K3" s="5" t="s">
-        <v>356</v>
+        <v>361</v>
       </c>
       <c r="L3" s="5" t="s">
-        <v>366</v>
+        <v>371</v>
       </c>
       <c r="M3" s="5" t="s">
-        <v>369</v>
+        <v>374</v>
       </c>
       <c r="N3" s="5" t="s">
-        <v>372</v>
+        <v>377</v>
       </c>
     </row>
     <row r="4" spans="1:14">
@@ -56469,7 +56499,7 @@
       <c r="B1005" s="7"/>
     </row>
   </sheetData>
-  <sheetProtection password="DCB0" sheet="1" objects="1" scenarios="1"/>
+  <sheetProtection password="B4C7" sheet="1" objects="1" scenarios="1"/>
   <mergeCells count="1">
     <mergeCell ref="A4:N4"/>
   </mergeCells>

</xml_diff>

<commit_message>
Updated single-cell documentation link
</commit_message>
<xml_diff>
--- a/dist/checklists/xlsx/dwc/single_cell_manifest_version_dwc_sc_rnaseq_v0.4.xlsx
+++ b/dist/checklists/xlsx/dwc/single_cell_manifest_version_dwc_sc_rnaseq_v0.4.xlsx
@@ -2520,7 +2520,7 @@
       </c>
     </row>
   </sheetData>
-  <sheetProtection password="FED8" sheet="1" objects="1" scenarios="1"/>
+  <sheetProtection password="A6E8" sheet="1" objects="1" scenarios="1"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
@@ -5601,7 +5601,7 @@
       <c r="A1005" s="7"/>
     </row>
   </sheetData>
-  <sheetProtection password="971B" sheet="1" objects="1" scenarios="1"/>
+  <sheetProtection password="EEF2" sheet="1" objects="1" scenarios="1"/>
   <mergeCells count="1">
     <mergeCell ref="A4:E4"/>
   </mergeCells>
@@ -8808,7 +8808,7 @@
       <c r="A1005" s="7"/>
     </row>
   </sheetData>
-  <sheetProtection password="DB6D" sheet="1" objects="1" scenarios="1"/>
+  <sheetProtection password="F6BF" sheet="1" objects="1" scenarios="1"/>
   <mergeCells count="1">
     <mergeCell ref="A4:O4"/>
   </mergeCells>
@@ -11884,7 +11884,7 @@
       <c r="A1005" s="7"/>
     </row>
   </sheetData>
-  <sheetProtection password="CD45" sheet="1" objects="1" scenarios="1"/>
+  <sheetProtection password="C343" sheet="1" objects="1" scenarios="1"/>
   <mergeCells count="1">
     <mergeCell ref="A4:D4"/>
   </mergeCells>
@@ -12003,7 +12003,7 @@
       <c r="H4" s="6"/>
     </row>
   </sheetData>
-  <sheetProtection password="FF9A" sheet="1" objects="1" scenarios="1"/>
+  <sheetProtection password="DC34" sheet="1" objects="1" scenarios="1"/>
   <mergeCells count="1">
     <mergeCell ref="A4:H4"/>
   </mergeCells>
@@ -18158,7 +18158,7 @@
       <c r="D1005" s="7"/>
     </row>
   </sheetData>
-  <sheetProtection password="F7C1" sheet="1" objects="1" scenarios="1"/>
+  <sheetProtection password="9DB6" sheet="1" objects="1" scenarios="1"/>
   <mergeCells count="1">
     <mergeCell ref="A4:K4"/>
   </mergeCells>
@@ -22369,7 +22369,7 @@
       <c r="B1005" s="7"/>
     </row>
   </sheetData>
-  <sheetProtection password="AF3D" sheet="1" objects="1" scenarios="1"/>
+  <sheetProtection password="F7B0" sheet="1" objects="1" scenarios="1"/>
   <mergeCells count="1">
     <mergeCell ref="A4:P4"/>
   </mergeCells>
@@ -28541,7 +28541,7 @@
       <c r="D1005" s="7"/>
     </row>
   </sheetData>
-  <sheetProtection password="BBD1" sheet="1" objects="1" scenarios="1"/>
+  <sheetProtection password="A066" sheet="1" objects="1" scenarios="1"/>
   <mergeCells count="1">
     <mergeCell ref="A4:K4"/>
   </mergeCells>
@@ -28665,7 +28665,7 @@
       <c r="H4" s="6"/>
     </row>
   </sheetData>
-  <sheetProtection password="82C8" sheet="1" objects="1" scenarios="1"/>
+  <sheetProtection password="9F1C" sheet="1" objects="1" scenarios="1"/>
   <mergeCells count="1">
     <mergeCell ref="A4:H4"/>
   </mergeCells>
@@ -32466,7 +32466,7 @@
       <c r="A1005" s="7"/>
     </row>
   </sheetData>
-  <sheetProtection password="8C47" sheet="1" objects="1" scenarios="1"/>
+  <sheetProtection password="8F2B" sheet="1" objects="1" scenarios="1"/>
   <mergeCells count="1">
     <mergeCell ref="A4:H4"/>
   </mergeCells>
@@ -36556,7 +36556,7 @@
       <c r="B1005" s="7"/>
     </row>
   </sheetData>
-  <sheetProtection password="D8D6" sheet="1" objects="1" scenarios="1"/>
+  <sheetProtection password="901C" sheet="1" objects="1" scenarios="1"/>
   <mergeCells count="1">
     <mergeCell ref="A4:E4"/>
   </mergeCells>
@@ -40712,7 +40712,7 @@
       <c r="B1005" s="7"/>
     </row>
   </sheetData>
-  <sheetProtection password="92BB" sheet="1" objects="1" scenarios="1"/>
+  <sheetProtection password="A20C" sheet="1" objects="1" scenarios="1"/>
   <mergeCells count="1">
     <mergeCell ref="A4:K4"/>
   </mergeCells>
@@ -46908,7 +46908,7 @@
       <c r="D1005" s="7"/>
     </row>
   </sheetData>
-  <sheetProtection password="E1A5" sheet="1" objects="1" scenarios="1"/>
+  <sheetProtection password="815C" sheet="1" objects="1" scenarios="1"/>
   <mergeCells count="1">
     <mergeCell ref="A4:N4"/>
   </mergeCells>
@@ -52279,7 +52279,7 @@
       <c r="C1005" s="7"/>
     </row>
   </sheetData>
-  <sheetProtection password="C639" sheet="1" objects="1" scenarios="1"/>
+  <sheetProtection password="F775" sheet="1" objects="1" scenarios="1"/>
   <mergeCells count="1">
     <mergeCell ref="A4:AD4"/>
   </mergeCells>
@@ -56499,7 +56499,7 @@
       <c r="B1005" s="7"/>
     </row>
   </sheetData>
-  <sheetProtection password="B4C7" sheet="1" objects="1" scenarios="1"/>
+  <sheetProtection password="AEAD" sheet="1" objects="1" scenarios="1"/>
   <mergeCells count="1">
     <mergeCell ref="A4:N4"/>
   </mergeCells>

</xml_diff>